<commit_message>
sube mediciones del dia 1/4, y script de prueba de delay
</commit_message>
<xml_diff>
--- a/codigo/firmware/Controlador/Prototipo/pines.xlsx
+++ b/codigo/firmware/Controlador/Prototipo/pines.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView minimized="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="109">
   <si>
     <t>PC9</t>
   </si>
@@ -308,6 +308,39 @@
   </si>
   <si>
     <t>GRoUND</t>
+  </si>
+  <si>
+    <t>IN0</t>
+  </si>
+  <si>
+    <t>IN4</t>
+  </si>
+  <si>
+    <t>IN5</t>
+  </si>
+  <si>
+    <t>IN6</t>
+  </si>
+  <si>
+    <t>IN7</t>
+  </si>
+  <si>
+    <t>IN8</t>
+  </si>
+  <si>
+    <t>IN10</t>
+  </si>
+  <si>
+    <t>IN11</t>
+  </si>
+  <si>
+    <t>IN14</t>
+  </si>
+  <si>
+    <t>CANAL ADC</t>
+  </si>
+  <si>
+    <t>IN1</t>
   </si>
 </sst>
 </file>
@@ -461,7 +494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -563,11 +596,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -876,22 +918,23 @@
   <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2">
@@ -1460,8 +1503,11 @@
       <c r="F30" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="G30" s="43" t="s">
+      <c r="G30" s="45" t="s">
         <v>96</v>
+      </c>
+      <c r="H30" s="47" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1477,8 +1523,11 @@
       <c r="F31" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="G31" s="40" t="s">
+      <c r="G31" s="44" t="s">
         <v>85</v>
+      </c>
+      <c r="H31" s="40" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1494,16 +1543,22 @@
       <c r="F32" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="G32" s="40" t="s">
+      <c r="G32" s="44" t="s">
         <v>86</v>
+      </c>
+      <c r="H32" s="40" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F33" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="G33" s="40" t="s">
+      <c r="G33" s="44" t="s">
         <v>83</v>
+      </c>
+      <c r="H33" s="40" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1522,8 +1577,11 @@
       <c r="F34" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="G34" s="40" t="s">
+      <c r="G34" s="44" t="s">
         <v>87</v>
+      </c>
+      <c r="H34" s="40" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -1542,8 +1600,11 @@
       <c r="F35" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="G35" s="40" t="s">
+      <c r="G35" s="44" t="s">
         <v>89</v>
+      </c>
+      <c r="H35" s="40" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1562,8 +1623,11 @@
       <c r="F36" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="G36" s="40" t="s">
+      <c r="G36" s="44" t="s">
         <v>90</v>
+      </c>
+      <c r="H36" s="40" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -1582,8 +1646,11 @@
       <c r="F37" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="G37" s="40" t="s">
+      <c r="G37" s="44" t="s">
         <v>93</v>
+      </c>
+      <c r="H37" s="40" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -1602,8 +1669,11 @@
       <c r="F38" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="G38" s="40" t="s">
+      <c r="G38" s="44" t="s">
         <v>92</v>
+      </c>
+      <c r="H38" s="40" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -1622,8 +1692,11 @@
       <c r="F39" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="G39" s="40" t="s">
+      <c r="G39" s="44" t="s">
         <v>84</v>
+      </c>
+      <c r="H39" s="40" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1642,8 +1715,11 @@
       <c r="F40" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="G40" s="41" t="s">
+      <c r="G40" s="46" t="s">
         <v>94</v>
+      </c>
+      <c r="H40" s="41" t="s">
+        <v>106</v>
       </c>
       <c r="I40" s="37"/>
     </row>

</xml_diff>